<commit_message>
feat: Establish Crisp-Inspired Growth Marketing & Aspirational Referral Playbook (File 47)
</commit_message>
<xml_diff>
--- a/10_Outreach_&_Relationship_Banking/Georgia_B2B_Outreach_&_Referral_Directory.xlsx
+++ b/10_Outreach_&_Relationship_Banking/Georgia_B2B_Outreach_&_Referral_Directory.xlsx
@@ -541,16 +541,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="314" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="41" customWidth="1" min="5" max="5"/>
+    <col width="57" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
     <col width="47" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -812,7 +812,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>5 Programs</t>
+          <t>6 Programs</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -833,6 +833,43 @@
       <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Track D: Split Booster / On-Site Civil Upgrades</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>7. Aspirational Referrals</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Landowners, Masterminds &amp; B2B Partners</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>4 Tiers</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Crisp-inspired high-stakes gamified referral framework</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Premium lifestyle &amp; high-status rewards</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>File 47: High-Growth Marketing Playbook</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>High-Stakes Aspirational Incentives / Patagonia Excursion</t>
         </is>
       </c>
     </row>
@@ -27318,7 +27355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -27552,6 +27589,43 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="68" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>LO-06</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Track 4: Patagonia Sweepstakes</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Entry into the Annual Grand Legacy Sweepstakes (one entry per successfully executed JV contract).</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Live drawing held on Dec 15th at the Annual Legacy Stream Summit. Luxury travel package fully managed by Developer.</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>7-day ultra-luxury guided fly-fishing excursion for two to Patagonia, Argentina (Estancia, guides, float trips, full outfitting gear).</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>30,000 USD (Value per drawing prize experience)</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>Underwritten under B2B marketing budget; Developer issues IRS Form 1099-MISC to winning partner.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>